<commit_message>
KUEHNE NAGEL: join PO numbers with "," (no space)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_samples/KUEHNE_NAGEL/sample3_ref.xlsx
+++ b/test_samples/KUEHNE_NAGEL/sample3_ref.xlsx
@@ -765,7 +765,7 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I5" s="5" t="n">
@@ -842,7 +842,7 @@
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I6" s="5" t="n">
@@ -919,7 +919,7 @@
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I7" s="5" t="n">
@@ -996,7 +996,7 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I8" s="5" t="n">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I9" s="5" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I10" s="5" t="n">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I11" s="5" t="n">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I12" s="5" t="n">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I13" s="5" t="n">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I14" s="5" t="n">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>4501208511, 4501208622, 4501208514, 4501208502, 4501208568, 4501208620, 4501208509</t>
+          <t>4501208511,4501208622,4501208514,4501208502,4501208568,4501208620,4501208509</t>
         </is>
       </c>
       <c r="I15" s="5" t="n">

</xml_diff>